<commit_message>
Umbral único de recomendación ±5% (COMPRAR); portada y presentación con las mismas cifras oficiales; presentación sin pies de fuente y con franja de cifras, índice y distintivo de recomendación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3Z6Fw74B8ffLJq5CxcxMa
</commit_message>
<xml_diff>
--- a/entregables/ValuFlow_Soriana_Modelo_2026-10-19.xlsx
+++ b/entregables/ValuFlow_Soriana_Modelo_2026-10-19.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="1316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="1321">
   <si>
     <t>Valuación de Organización Soriana, S.A.B. de C.V.: DCF, múltiplos y transacciones precedentes</t>
   </si>
@@ -141,7 +141,7 @@
     <t>Recomendación</t>
   </si>
   <si>
-    <t>MANTENER (potencial +7.3% frente a $33.48)</t>
+    <t>COMPRAR (potencial +7.3% frente a $33.48)</t>
   </si>
   <si>
     <t>WACC / Ke / g</t>
@@ -1080,10 +1080,10 @@
     <t>Recomendación de la app</t>
   </si>
   <si>
-    <t>MANTENER</t>
-  </si>
-  <si>
-    <t>Precio objetivo = valuación combinada; COMPRAR si el potencial supera +10%, VENDER si es menor que −10% (hoja Transacciones SDC §7).</t>
+    <t>COMPRAR</t>
+  </si>
+  <si>
+    <t>Precio objetivo = valuación combinada; COMPRAR si el potencial supera +5%, VENDER si es menor que −5% (hoja Transacciones SDC §7).</t>
   </si>
   <si>
     <t>1. Resumen ejecutivo</t>
@@ -3321,7 +3321,7 @@
     <t>Umbral de compra / venta</t>
   </si>
   <si>
-    <t>+10% / −10%</t>
+    <t>+5% / −5%</t>
   </si>
   <si>
     <t>Rango de valor razonable</t>
@@ -3948,6 +3948,21 @@
     <t>14</t>
   </si>
   <si>
+    <t>Había dos umbrales: ±15% para la lectura del DCF (Proyección Final B155) y ±10% para la recomendación oficial (Transacciones SDC §7).</t>
+  </si>
+  <si>
+    <t>Dos reglas distintas podían dar recomendaciones diferentes.</t>
+  </si>
+  <si>
+    <t>Un solo umbral de ±5%: Transacciones SDC §7 (COMPRAR / VENDER) y B155 vinculado a esa celda.</t>
+  </si>
+  <si>
+    <t>Validación y extractor leen el mismo umbral.</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
     <t>Revisado, sin cambio</t>
   </si>
   <si>
@@ -3960,7 +3975,7 @@
     <t>Recálculo independiente y controles 23–32.</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>Fechas</t>
@@ -13970,7 +13985,7 @@
         <v>95</v>
       </c>
       <c r="B27" s="10">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C27" t="s">
         <v>54</v>
@@ -13984,7 +13999,7 @@
         <v>97</v>
       </c>
       <c r="B28" s="10">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="C28" t="s">
         <v>54</v>
@@ -14850,7 +14865,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -15974,18 +15989,18 @@
         <v>1304</v>
       </c>
       <c r="B66" s="35" t="s">
-        <v>341</v>
-      </c>
-      <c r="C66" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="C66" s="34" t="s">
+        <v>1299</v>
+      </c>
+      <c r="D66" s="34" t="s">
         <v>1305</v>
       </c>
-      <c r="D66" s="34" t="s">
+      <c r="E66" s="34" t="s">
         <v>1306</v>
       </c>
-      <c r="E66" s="35" t="s">
-        <v>386</v>
-      </c>
-      <c r="F66" s="35" t="s">
+      <c r="F66" s="34" t="s">
         <v>1307</v>
       </c>
       <c r="G66" s="34" t="s">
@@ -15997,32 +16012,55 @@
         <v>1309</v>
       </c>
       <c r="B67" s="33" t="s">
+        <v>341</v>
+      </c>
+      <c r="C67" s="33" t="s">
         <v>1310</v>
-      </c>
-      <c r="C67" s="33" t="s">
-        <v>1305</v>
       </c>
       <c r="D67" s="32" t="s">
         <v>1311</v>
       </c>
       <c r="E67" s="33" t="s">
+        <v>386</v>
+      </c>
+      <c r="F67" s="33" t="s">
         <v>1312</v>
       </c>
-      <c r="F67" s="32" t="s">
+      <c r="G67" s="32" t="s">
         <v>1313</v>
       </c>
-      <c r="G67" s="33" t="s">
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="34" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B68" s="35" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C68" s="35" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D68" s="34" t="s">
+        <v>1316</v>
+      </c>
+      <c r="E68" s="35" t="s">
+        <v>1317</v>
+      </c>
+      <c r="F68" s="34" t="s">
+        <v>1318</v>
+      </c>
+      <c r="G68" s="35" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" s="42" t="s">
-        <v>1314</v>
-      </c>
-    </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" s="2" t="s">
-        <v>1315</v>
+      <c r="A69" s="42" t="s">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>1320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>